<commit_message>
Merged files together so far
</commit_message>
<xml_diff>
--- a/your-project/Resources/Avg cost of living.xlsx
+++ b/your-project/Resources/Avg cost of living.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mattymrc/Desktop/Ironhack/Projects/Project-Week-2-Lisbon/your-project/Resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEAA0722-3256-A84D-AEBE-F4EEC3F6165B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1ED76F1-8929-B348-A7B4-300DC90A6EE0}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="460" windowWidth="28800" windowHeight="16280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,9 +20,7 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -101,13 +99,13 @@
     <t>Benfica</t>
   </si>
   <si>
-    <t>Santo Antão</t>
-  </si>
-  <si>
     <t>Current Freguesias</t>
   </si>
   <si>
     <t>average rent in euro</t>
+  </si>
+  <si>
+    <t>Santo António</t>
   </si>
 </sst>
 </file>
@@ -957,10 +955,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s">
         <v>24</v>
-      </c>
-      <c r="B1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -1133,7 +1131,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B23">
         <v>386.26</v>

</xml_diff>